<commit_message>
updated ParentID output, improved export functionality for testing, updated README.md
</commit_message>
<xml_diff>
--- a/requirement_documents/Tracing_Examples/Level4Reqs.xlsx
+++ b/requirement_documents/Tracing_Examples/Level4Reqs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\christopher\RM\requirement_documents\Tracing_Examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C26EF4-A66E-4098-A854-F671F531342C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{474432F2-9D5A-46E7-8284-E931714B48C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="67095" yWindow="10440" windowWidth="19410" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="49">
   <si>
     <t>ID</t>
   </si>
@@ -169,6 +169,9 @@
   </si>
   <si>
     <t>Verify via command tests.</t>
+  </si>
+  <si>
+    <t>REQ-MIS-004</t>
   </si>
 </sst>
 </file>
@@ -529,7 +532,7 @@
     </row>
     <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
added transforms of certain columns with cfg for special files that split the requirement name into several columns
</commit_message>
<xml_diff>
--- a/requirement_documents/Tracing_Examples/Level4Reqs.xlsx
+++ b/requirement_documents/Tracing_Examples/Level4Reqs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\christopher\RM\requirement_documents\Tracing_Examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{474432F2-9D5A-46E7-8284-E931714B48C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AA63B2-4A80-4B89-A70D-FD6C961D6F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67095" yWindow="10440" windowWidth="19410" windowHeight="10545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="47880" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -120,9 +120,6 @@
     <t>The processing unit shall support required communication interfaces.</t>
   </si>
   <si>
-    <t>E.g., SpaceWire.</t>
-  </si>
-  <si>
     <t>Verify via interface validation.</t>
   </si>
   <si>
@@ -172,6 +169,9 @@
   </si>
   <si>
     <t>REQ-MIS-004</t>
+  </si>
+  <si>
+    <t>Deleted</t>
   </si>
 </sst>
 </file>
@@ -532,7 +532,7 @@
     </row>
     <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
@@ -613,10 +613,10 @@
         <v>30</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>17</v>
@@ -627,19 +627,19 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>17</v>
@@ -650,19 +650,19 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
         <v>38</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>39</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>40</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>41</v>
-      </c>
-      <c r="F7" t="s">
-        <v>42</v>
       </c>
       <c r="G7" t="s">
         <v>17</v>
@@ -673,19 +673,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
         <v>43</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>44</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>45</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>46</v>
-      </c>
-      <c r="F8" t="s">
-        <v>47</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>

</xml_diff>